<commit_message>
docs(spec): expand specification sheets to 5+ rows and update validation hashes
</commit_message>
<xml_diff>
--- a/specification/Nhom11_SecureGate_IoT_Gateway_Spec.xlsx
+++ b/specification/Nhom11_SecureGate_IoT_Gateway_Spec.xlsx
@@ -45,7 +45,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -56,6 +56,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="001F4E79"/>
         <bgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+        <bgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F5F8"/>
+        <bgColor rgb="00F2F5F8"/>
       </patternFill>
     </fill>
   </fills>
@@ -85,12 +97,21 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -462,7 +483,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="58" customWidth="1" min="2" max="2"/>
+    <col width="65" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -490,12 +511,12 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>Bộ phân tích cú pháp gói tin nhị phân và kiểm soát truy cập SecureGate IoT Gateway (Giao thức IGW1: Header 16-byte, Checksum 32-bit, Registration type=0x01, Unlock type=0x02). Nhóm 11 - Lưu Đức Hiệp &amp; Hà Nguyễn Trúc Linh.</t>
         </is>
@@ -512,16 +533,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
     <col width="35" customWidth="1" min="2" max="2"/>
-    <col width="58" customWidth="1" min="3" max="3"/>
-    <col width="58" customWidth="1" min="4" max="4"/>
-    <col width="58" customWidth="1" min="5" max="5"/>
-    <col width="58" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="65" customWidth="1" min="3" max="3"/>
+    <col width="65" customWidth="1" min="4" max="4"/>
+    <col width="65" customWidth="1" min="5" max="5"/>
+    <col width="65" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -572,7 +593,7 @@
           <t>REQ-SG-01, REQ-SG-02</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="5" t="inlineStr">
         <is>
           <t>Kiểm chứng xung đột đồng thời giữa xử lý Registration và Unlock</t>
         </is>
@@ -582,14 +603,14 @@
           <t>Hệ thống ở trạng thái gw_idle</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" s="5" t="inlineStr">
         <is>
           <t>Tiến trình nhận gói Registration kích hoạt trạng thái rx_reg_packet
 Đồng thời tiến trình Unlock kích hoạt trạng thái rx_unlock_packet
 Kiểm chứng mô hình Kripke bằng thuật toán Model Checking</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" s="5" t="inlineStr">
         <is>
           <t>Mô hình chuyển vào trạng thái gw_race_hazard làm thuộc tính AG(!violation) bị SAI (phát hiện phản ví dụ)</t>
         </is>
@@ -601,38 +622,38 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>TC-SG-02</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>REQ-SG-03</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>REQ-SG-03, CON-SG-02</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>Kiểm thử lỗi tràn bộ đệm khi device_id trong gói tin nhị phân vượt quá 16 bytes</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>Hàm parse_securegate_device_id() sinh từ đặc tả với bug=buffer-overflow</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>Sinh mã nguồn C cho hàm parse_securegate_device_id()
 Chạy công cụ phân tích tĩnh check_c_source()</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F3" s="4" t="inlineStr">
         <is>
           <t>Phát hiện cảnh báo dangerous-function (CWE-120/121) do hàm strcpy sao chép vào buffer 16 bytes không kiểm tra biên</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -644,28 +665,28 @@
           <t>TC-SG-03</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>REQ-SG-04, REQ-SG-05, REQ-SG-06</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>Kiểm tra chu kỳ cấp phát và giải phóng tài nguyên bộ nhớ C</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>Các hàm log_securegate_audit_event, terminate_securegate_session, cleanup_stream_buffer đã được sinh mã C</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>Gộp toàn bộ mã C của các hàm quản lý tài nguyên
 Thực thi check_c_source() trên khối mã gộp</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>Phát hiện đủ 3 lớp lỗ hổng bộ nhớ: Rò rỉ bộ nhớ (CWE-401), Giải phóng trùng lặp (CWE-415), và Truy cập sau giải phóng (CWE-416)</t>
         </is>
@@ -677,37 +698,37 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>TC-SG-04</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>REQ-SG-07</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>Kiểm chứng nguy cơ tràn số nguyên 32-bit trong bộ cộng dồn checksum gói tin</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>Hai biến header_checksum và payload_checksum không âm có tổng &gt; 2 tỷ</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>Thực thi kiểm tra check_int32_overflow() bằng Z3 SMT Solver trên biểu thức header_checksum + payload_checksum</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>Z3 Solver trả về kết quả SAT cùng nghiệm phản ví dụ chứng minh biểu thức vượt giới hạn INT32_MAX</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -724,22 +745,22 @@
           <t>REQ-SG-08</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>Fuzzing hộp đen hàm tính toán tỷ lệ rớt gói calculate_gateway_drop_ratio</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>Hàm Python calculate_gateway_drop_ratio(received_packets, dropped_packets) sinh từ đặc tả</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>Chạy blackbox_fuzz() ngẫu nhiên 300 lượt thử</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="F6" s="5" t="inlineStr">
         <is>
           <t>Tìm thấy ít nhất 1 đầu vào có dropped_packets=0 kích hoạt crash ZeroDivisionError (CWE-369)</t>
         </is>
@@ -751,37 +772,115 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>TC-SG-06</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>REQ-SG-09</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>REQ-SG-09, CON-SG-03</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>Kiểm thử Concolic giải ngược cặp mã mở khóa bí mật 32-bit (7421, 3390)</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>Hàm Python verify_securegate_unlock_guard(unlock_a, unlock_b) với magic values=(7421, 3390)</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>Chạy concolic_fuzz() với ngân sách tối đa 15 vòng lặp</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="F7" s="4" t="inlineStr">
         <is>
           <t>Thuật toán Concolic giải hệ phương trình đường đi thành công và tìm ra đúng cặp (7421, 3390) chỉ trong &lt;= 15 lần thử</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>TC-SG-07</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>NFR-SG-01, NFR-SG-02, CON-SG-01</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Kiểm định thông lượng phân tích gói tin và độ trễ xác thực checksum</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Phần cứng máy chủ IoT tiêu chuẩn, tập dữ liệu seed corpus 500 gói tin IGW1</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Nạp tập seed corpus 500 gói tin nhị phân IGW1 vào parser
+Đo tổng thời gian phân tích và xác thực checksum toàn vẹn
+Tính toán thông lượng trung bình (packets/sec) và độ trễ xử lý (ms/packet)</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>Hệ thống đạt thông lượng &gt;= 500 gói/s (NFR-SG-01) và độ trễ xử lý &lt; 5ms (NFR-SG-02), gói tin tuân thủ CON-SG-01</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>TC-SG-08</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>NFR-SG-04, CON-SG-04, CON-SG-05</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Kiểm tra giới hạn dung lượng RAM và khả năng chịu tải gói tin cực đại</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Môi trường thực thi bộ parser biên dịch bằng GCC theo chuẩn ISO C99/C11</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Sinh gói tin nhị phân có kích thước cực đại 65555 bytes theo CON-SG-04
+Đưa gói tin vào hàm parse_and_process() và đo đạc mức RAM cấp phát
+Giám sát toàn bộ chu kỳ sống để xác nhận không cấp phát trong ngắt ISR</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Dung lượng RAM tiêu thụ không vượt quá 2MB (NFR-SG-04), xử lý an toàn không xuất hiện lỗi tràn bộ nhớ</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
@@ -801,10 +900,10 @@
   <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="58" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="65" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -835,7 +934,7 @@
           <t>REQ-SG-01</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="5" t="inlineStr">
         <is>
           <t>Tiến trình xử lý gói tin Registration và tiến trình xử lý Unlock không được đồng thời can thiệp vào vùng đệm chia sẻ của gateway (Mutual Exclusion)</t>
         </is>
@@ -852,22 +951,22 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>REQ-SG-02</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>Bộ phân tích cú pháp SecureGate không được rơi vào trạng thái bế tắc (deadlock) khi các tiến trình luân phiên xử lý gói tin nhị phân</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>liveness</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -879,7 +978,7 @@
           <t>REQ-SG-03</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Hàm parse_securegate_device_id() khi phân tích chuỗi device_id từ payload nhị phân không được gây tràn bộ đệm ngăn xếp (Stack Buffer Overflow - CWE-121)</t>
         </is>
@@ -896,22 +995,22 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>REQ-SG-04</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Hàm log_securegate_audit_event() phải giải phóng toàn bộ bộ nhớ động đã cấp phát sau khi ghi log gói tin để tránh cạn kiệt tài nguyên (CWE-401)</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>memory</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -923,7 +1022,7 @@
           <t>REQ-SG-05</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>Hàm terminate_securegate_session() khi đóng kênh kết nối client không được giải phóng cùng một con trỏ nhiều lần (Double-Free - CWE-415)</t>
         </is>
@@ -940,22 +1039,22 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>REQ-SG-06</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>Hàm cleanup_stream_buffer() không được ghi dữ liệu vào vùng đệm gói tin sau khi bộ nhớ đã được giải phóng (Use-After-Free - CWE-416)</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>memory</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -967,7 +1066,7 @@
           <t>REQ-SG-07</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Bộ tích lũy tổng checksum số học securegate_checksum_accumulator không được gây hiện tượng tràn số nguyên 32-bit có dấu (CWE-190)</t>
         </is>
@@ -984,22 +1083,22 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>REQ-SG-08</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>Hàm tính toán tỷ lệ mất gói calculate_gateway_drop_ratio() không được gây crash không kiểm soát khi số lượng gói tin rớt bằng 0 (CWE-369)</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>functional</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -1011,7 +1110,7 @@
           <t>REQ-SG-09</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>Cơ chế mở khóa khẩn cấp verify_securegate_unlock_guard() với cặp mã 16-bit (7421, 3390) phải được kiểm thử tự động bằng kỹ thuật Fuzzing thông minh</t>
         </is>
@@ -1038,12 +1137,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="58" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="65" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1069,7 +1168,7 @@
           <t>NFR-SG-01</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="5" t="inlineStr">
         <is>
           <t>Hệ thống SecureGate Gateway phải phân tích cú pháp tối thiểu 500 gói tin nhị phân IGW1 mỗi giây trên phần cứng tiêu chuẩn</t>
         </is>
@@ -1081,17 +1180,17 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>NFR-SG-02</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>Thời gian phân tích hợp lệ và xác thực checksum cho một gói tin nhị phân kích thước dưới 1KB phải hoàn thành trong dưới 5ms</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -1103,7 +1202,7 @@
           <t>NFR-SG-03</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Nhật ký kiểm toán sự kiện an ninh nhị phân phải được ghi đồng bộ, bảo đảm tính toàn vẹn ngay cả khi luồng ghi log bị ngắt đột ngột</t>
         </is>
@@ -1111,6 +1210,40 @@
       <c r="C4" s="2" t="inlineStr">
         <is>
           <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>NFR-SG-04</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Mức tiêu thụ bộ nhớ RAM tối đa của bộ phân tích cú pháp không vượt quá 2MB trong suốt vòng đời xử lý gói tin</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>NFR-SG-05</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Tỷ lệ rớt gói tin ngoài ý muốn do nghẽn hàng đợi hoặc xử lý phân tích cú pháp không vượt quá 0.01% tổng lưu lượng</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
     </row>
@@ -1125,12 +1258,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="58" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="65" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1156,7 +1289,7 @@
           <t>CON-SG-01</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="5" t="inlineStr">
         <is>
           <t>Gói tin mạng phải tuân thủ nghiêm ngặt cấu trúc nhị phân IGW1: Header 16 bytes, Checksum 4 bytes ở cuối gói, định dạng số nguyên little-endian</t>
         </is>
@@ -1168,17 +1301,17 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>CON-SG-02</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>Mã nhận diện thiết bị device_id trong gói tin Registration có độ dài tối đa 16 ký tự, mã hóa hoàn toàn bằng ký tự ASCII in được (0x20 - 0x7E)</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -1190,12 +1323,46 @@
           <t>CON-SG-03</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Mã mở khóa khẩn cấp SecureGate phải bao gồm đúng 2 trường số nguyên không dấu 16-bit (unlock_a, unlock_b) nằm trong header</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>CON-SG-04</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Tổng chiều dài toàn bộ gói tin nhị phân (header + payload + checksum) không được vượt quá giới hạn 65555 bytes</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>CON-SG-05</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Toàn bộ mã nguồn C xử lý phân tích cú pháp phải tuân thủ tiêu chuẩn ISO C99/C11, nghiêm cấm cấp phát động trong ngắt ISR</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -1216,7 +1383,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
     <col width="48" customWidth="1" min="3" max="3"/>
     <col width="35" customWidth="1" min="4" max="4"/>
   </cols>
@@ -1256,28 +1423,28 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
+          <t>safe, ready</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
         <is>
           <t>rx_reg_packet, rx_unlock_packet</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>rx_reg_packet</t>
         </is>
       </c>
-      <c r="B3" s="2" t="n"/>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="B3" s="3" t="n"/>
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>reg_processing</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>gw_idle, gw_race_hazard</t>
         </is>
@@ -1302,18 +1469,18 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>gw_race_hazard</t>
         </is>
       </c>
-      <c r="B5" s="2" t="n"/>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="B5" s="3" t="n"/>
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>reg_processing, unlock_processing, violation</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>gw_idle</t>
         </is>
@@ -1330,10 +1497,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="37" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1351,7 +1518,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>EF(reg_processing)</t>
         </is>
@@ -1361,6 +1528,20 @@
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>EF(unlock_processing)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>AG(reg_processing -&gt; AF(safe))</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>AG(unlock_processing -&gt; AF(safe))</t>
         </is>
       </c>
     </row>
@@ -1375,10 +1556,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="21" customWidth="1" min="1" max="1"/>
     <col width="21" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -1403,6 +1584,54 @@
       <c r="B2" s="2" t="inlineStr">
         <is>
           <t>unlock_processing</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>reg_processing</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>safe</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>unlock_processing</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>safe</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>violation</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>safe</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>violation</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>ready</t>
         </is>
       </c>
     </row>
@@ -1421,7 +1650,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="37" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
@@ -1509,34 +1738,34 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>log_securegate_audit_event</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>alloc_release</t>
         </is>
       </c>
-      <c r="D3" s="2" t="n"/>
-      <c r="E3" s="2" t="n">
+      <c r="D3" s="3" t="n"/>
+      <c r="E3" s="3" t="n">
         <v>32</v>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>memory-leak</t>
         </is>
       </c>
-      <c r="G3" s="2" t="n">
+      <c r="G3" s="3" t="n">
         <v>1234</v>
       </c>
-      <c r="H3" s="2" t="n">
+      <c r="H3" s="3" t="n">
         <v>5678</v>
       </c>
     </row>
@@ -1573,34 +1802,34 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>cleanup_stream_buffer</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>alloc_release</t>
         </is>
       </c>
-      <c r="D5" s="2" t="n"/>
-      <c r="E5" s="2" t="n">
+      <c r="D5" s="3" t="n"/>
+      <c r="E5" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>use-after-free</t>
         </is>
       </c>
-      <c r="G5" s="2" t="n">
+      <c r="G5" s="3" t="n">
         <v>1234</v>
       </c>
-      <c r="H5" s="2" t="n">
+      <c r="H5" s="3" t="n">
         <v>5678</v>
       </c>
     </row>
@@ -1620,7 +1849,7 @@
           <t>divide</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>received_packets, dropped_packets</t>
         </is>
@@ -1637,34 +1866,34 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>verify_securegate_unlock_guard</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>python</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>magic_value</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>unlock_a, unlock_b</t>
         </is>
       </c>
-      <c r="E7" s="2" t="n">
+      <c r="E7" s="3" t="n">
         <v>16</v>
       </c>
-      <c r="F7" s="2" t="n"/>
-      <c r="G7" s="2" t="n">
+      <c r="F7" s="3" t="n"/>
+      <c r="G7" s="3" t="n">
         <v>7421</v>
       </c>
-      <c r="H7" s="2" t="n">
+      <c r="H7" s="3" t="n">
         <v>3390</v>
       </c>
     </row>
@@ -1679,12 +1908,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
     <col width="37" customWidth="1" min="2" max="2"/>
-    <col width="58" customWidth="1" min="3" max="3"/>
+    <col width="65" customWidth="1" min="3" max="3"/>
     <col width="38" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
@@ -1711,24 +1940,112 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="5" t="inlineStr">
         <is>
           <t>securegate_checksum_accumulator</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="5" t="inlineStr">
         <is>
           <t>header_checksum, payload_checksum</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="5" t="inlineStr">
         <is>
           <t>header_checksum &gt;= 0 and payload_checksum &gt;= 0 and header_checksum + payload_checksum &gt; 2000000000</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="5" t="inlineStr">
         <is>
           <t>header_checksum + payload_checksum</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>gateway_packet_counter</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>rx_packets, tx_packets</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>rx_packets &gt;= 0 and tx_packets &gt;= 0 and rx_packets + tx_packets &gt; 65535</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>rx_packets + tx_packets</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>gateway_telemetry_bytes</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>sensor_bytes, auth_bytes</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>sensor_bytes &gt;= 0 and auth_bytes &gt;= 0 and sensor_bytes + auth_bytes &gt; 2000000000</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>sensor_bytes + auth_bytes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>gateway_session_duration</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>active_duration, idle_duration</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>active_duration &gt;= 0 and idle_duration &gt;= 0 and active_duration + idle_duration &gt; 32767</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>active_duration + idle_duration</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>gateway_dropped_packets_counter</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>buffer_drops, auth_drops</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>buffer_drops &gt;= 0 and auth_drops &gt;= 0 and buffer_drops + auth_drops &gt; 65535</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>buffer_drops + auth_drops</t>
         </is>
       </c>
     </row>

</xml_diff>